<commit_message>
updated power analysis w t-test, added visuals
</commit_message>
<xml_diff>
--- a/data/clean/price_table.xlsx
+++ b/data/clean/price_table.xlsx
@@ -21,13 +21,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -46,12 +49,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -421,64 +454,64 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Bulldega</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Durham Co-op</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Food Lion</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Gazelle</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Harris Teeter</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Whole Foods</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>n_stores</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>control_price</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>beer</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Blue Ribbon | Narragansett, 12 pk lager cans</t>
         </is>
@@ -507,7 +540,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Budweiser | 25 oz bud light</t>
         </is>
@@ -532,7 +566,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Pisgah | 6 pack pale ale</t>
         </is>
@@ -555,7 +590,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="1" t="n"/>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Ponysaurus | Biere de garde, 6 pk</t>
         </is>
@@ -580,7 +616,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Sierra Nevada | Pale ale 12 pk</t>
         </is>
@@ -609,12 +646,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>dairy</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>Organic Valley | Organic 2%, 64 fz</t>
         </is>
@@ -633,12 +670,12 @@
       <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>pantry</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Annie's | Classic cheddar pasta, 6 oz</t>
         </is>
@@ -657,7 +694,8 @@
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Annie's | Organic classic cheddar pasta, 6 oz</t>
         </is>
@@ -676,7 +714,8 @@
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="B10" t="inlineStr">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Jovial | Gf elbows</t>
         </is>
@@ -695,7 +734,8 @@
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="B11" t="inlineStr">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Jovial | Gf penne</t>
         </is>
@@ -714,12 +754,12 @@
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>Kettle brand | Sour cream and onion, 5 oz</t>
         </is>
@@ -738,12 +778,12 @@
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>snack bar</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Big Spoon | Apricot pepita</t>
         </is>
@@ -766,7 +806,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" t="inlineStr">
+      <c r="A14" s="1" t="n"/>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Big Spoon | Cherry chocolate</t>
         </is>
@@ -789,7 +830,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" t="inlineStr">
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Hu chocolate | Almond butter + puffed quinoa dark chocolate</t>
         </is>
@@ -808,7 +850,8 @@
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Kind | Dark chocolate mocha almond, 12 oz bar</t>
         </is>
@@ -835,7 +878,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" t="inlineStr">
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Kind | Peanut butter dark chocolate, 12 oz bar</t>
         </is>
@@ -862,7 +906,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" t="inlineStr">
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Luna | Bluberry, 1.69 oz</t>
         </is>
@@ -885,7 +930,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" t="inlineStr">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Luna | Lemon zest, 1.69</t>
         </is>
@@ -910,7 +956,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" t="inlineStr">
+      <c r="A20" s="1" t="n"/>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>RXBAR | Bluberry</t>
         </is>
@@ -937,7 +984,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" t="inlineStr">
+      <c r="A21" s="1" t="n"/>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>RXBAR | Peanut butter</t>
         </is>
@@ -983,59 +1031,59 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Bulldega</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Durham Co-op</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Food Lion</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Gazelle</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Harris Teeter</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Whole Foods</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>control_price</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>beer</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Blue Ribbon | Narragansett, 12 pk lager cans</t>
         </is>
@@ -1061,7 +1109,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Budweiser | 25 oz bud light</t>
         </is>
@@ -1083,7 +1132,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Pisgah | 6 pack pale ale</t>
         </is>
@@ -1103,7 +1153,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="1" t="n"/>
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Ponysaurus | Biere de garde, 6 pk</t>
         </is>
@@ -1125,7 +1176,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Sierra Nevada | Pale ale 12 pk</t>
         </is>
@@ -1151,12 +1203,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>dairy</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>Organic Valley | Organic 2%, 64 fz</t>
         </is>
@@ -1172,12 +1224,12 @@
       <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>pantry</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Annie's | Classic cheddar pasta, 6 oz</t>
         </is>
@@ -1193,7 +1245,8 @@
       <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="B9" t="inlineStr">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Annie's | Organic classic cheddar pasta, 6 oz</t>
         </is>
@@ -1209,7 +1262,8 @@
       <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="B10" t="inlineStr">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Jovial | Gf elbows</t>
         </is>
@@ -1225,7 +1279,8 @@
       <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="B11" t="inlineStr">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Jovial | Gf penne</t>
         </is>
@@ -1241,12 +1296,12 @@
       <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>snack</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>Kettle brand | Sour cream and onion, 5 oz</t>
         </is>
@@ -1262,12 +1317,12 @@
       <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>snack bar</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Big Spoon | Apricot pepita</t>
         </is>
@@ -1287,7 +1342,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" t="inlineStr">
+      <c r="A14" s="1" t="n"/>
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Big Spoon | Cherry chocolate</t>
         </is>
@@ -1307,7 +1363,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" t="inlineStr">
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Hu chocolate | Almond butter + puffed quinoa dark chocolate</t>
         </is>
@@ -1323,7 +1380,8 @@
       <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Kind | Dark chocolate mocha almond, 12 oz bar</t>
         </is>
@@ -1347,7 +1405,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" t="inlineStr">
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Kind | Peanut butter dark chocolate, 12 oz bar</t>
         </is>
@@ -1371,7 +1430,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" t="inlineStr">
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Luna | Bluberry, 1.69 oz</t>
         </is>
@@ -1391,7 +1451,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" t="inlineStr">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Luna | Lemon zest, 1.69</t>
         </is>
@@ -1413,7 +1474,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" t="inlineStr">
+      <c r="A20" s="1" t="n"/>
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>RXBAR | Bluberry</t>
         </is>
@@ -1437,7 +1499,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" t="inlineStr">
+      <c r="A21" s="1" t="n"/>
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>RXBAR | Peanut butter</t>
         </is>
@@ -1480,22 +1543,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>store</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>regular_price</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1634,112 +1697,112 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>brand</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>product</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>store</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>store_type</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>regular_price</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>sale_price</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>member_price</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>shelf</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>substitute</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>paid_price</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>found</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>storefront_price</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>amazon_total_wine_price</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>control_price</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>control_source</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>control_note</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>has_control</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>regular_premium_pct</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>paid_premium_pct</t>
         </is>
@@ -7572,42 +7635,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>brand</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>product</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>storefront_price</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>amazon_total_wine_price</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>control_price</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>control_source</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>control_note</t>
         </is>

</xml_diff>